<commit_message>
chore(data): Atualização das bases
</commit_message>
<xml_diff>
--- a/app/data/db_character_traits.xlsx
+++ b/app/data/db_character_traits.xlsx
@@ -858,14 +858,14 @@
     <t xml:space="preserve">
 - Uma vez a cada hora de jogo, você pode perceber hostilidade ou intenções violentas de alvos que possa ver.
 - Note também que o olhar não pode ser economizado. Você não pode jogar durante horas sem usar o olhar e, depois, usá-la várias vezes em seguida!
-- Uma vez por dia pode tornar uma manobra de ataque em ataque total, sem o redutor de perder sua manobra de defesa ativa.</t>
+- Uma vez por dia, ao realizar um Ataque Total, você mantém o direito a uma Defesa Ativa normalmente.</t>
   </si>
   <si>
     <t>OLHOS DE ASMODEUS</t>
   </si>
   <si>
     <t xml:space="preserve">
-- Uma vez a cada hora de jogo, você pode ganhar +1 em testes de Persuasão, Sedução ou Diplomacia.
+- Uma vez a cada hora de jogo, você pode ganhar +1 em testes de influência.
 - Note também que o olhar não pode ser economizado. Você não pode jogar durante horas sem usar o olhar e, depois, usá-la várias vezes em seguida!
 - Uma vez por dia pode descobrir o que uma pessoa mais deseja, momentaneamente, em uma interação social.</t>
   </si>
@@ -875,19 +875,18 @@
   <si>
     <t xml:space="preserve">
 - Uma vez por dia pode escolher um alvo que possa ver e:
-    - Cada golpe ou feitiço que acerte o alvo (que não seja aparado, bloqueado ou desviado), lhe concede um bônus de +1 para acertar este;
-    - Golpes consecutivos acumulam o bônus;
-    - Ao errar (ter seu golpe aparado, bloqueado ou desviado), aplica-se um redutor equivalente ao bônus que estava sobre o alvo;
-    - Ao errar não se pode ganhar bônus contra o alvo e o redutor permance até o fim do embate.
-- Esse efeito pode ser utilizado em um alvo por vez, mas pode ser utilizado em mais de um alvo caso o redutor seja aplicado contra algum deles.
-</t>
+    - Cada ataque ou feitiço que atinja o alvo (e não seja aparado, bloqueado, desviado ou resistido), lhe concede um bônus cumulativo de +1 em futuras ações contra este;
+    - O bônus aplica-se a ataques, feitiços, testes resistidos e testes de influência realizados contra o alvo;
+    - O bônus é cumulativo até o máximo de +5;
+    - Caso falhe em uma ação contra o alvo, perde todo o bônus acumulado e sofre um redutor equivalente até o fim do embate.
+- Esse efeito pode ser utilizado em apenas um alvo por vez, mas pode ser utilizado em um novo alvo após perder o bônus acumulado contra o anterior.</t>
   </si>
   <si>
     <t>OLHOS DE LEVIATHAN</t>
   </si>
   <si>
     <t xml:space="preserve">
-- Uma vez por dia pode copiar uma perícia ou feitiço de um alvo que você possa ver.
+- Uma vez por dia pode copiar uma perícia ou feitiço que tenha acabado de observar.
 - A perícia ou feitiço copiado tem seu nível de habilidade igual ao seu atributo de DX ou IQ, conforme o atributo deste, com +5 de bônus.
 - Essa habilidade pode ser utilizada apenas uma vez por dia.
 - Uma vez usada em combate a habilidade pode ser utilizada até o fim deste.</t>
@@ -899,16 +898,20 @@
     <t xml:space="preserve">
 - Uma vez a cada hora de jogo, você pode ganhar +1 em testes de Comércio ou Barganha.
 - Note também que o olhar não pode ser economizado. Você não pode jogar durante horas sem usar o olhar e, depois, usá-la várias vezes em seguida!
-- Uma vez por dia pode adcionar um bônus de +1 a uma jogada equivalente a cada 2000 moedas carregadas.</t>
+- Uma vez por dia, escolha um alvo que possua um item de valor, enquanto ela permanecer portando esse item, você recebe +2 em qualquer teste contra este.</t>
   </si>
   <si>
     <t>OLHOS DE LUCIFER</t>
   </si>
   <si>
     <t xml:space="preserve">
-- Uma vez a cada hora de jogo, você pode ganhar +1 em testes de Comércio ou Barganha.
-- Note também que o olhar não pode ser economizado. Você não pode jogar durante horas sem usar o olhar e, depois, usá-la várias vezes em seguida!
-- Uma vez por dia pode descobrir o menor preço que um mercador está disposto a pagar ou vender determinado item.</t>
+- Uma vez por dia pode escolher um alvo que possa ver e:
+    - Sempre que obtiver sucesso contra o alvo em um teste resistido, ataque ou influência social, recebe um bônus cumulativo de +1 em futuras ações contra este;
+    - O bônus aplica-se a ataques, feitiços, testes resistidos e testes de influência realizados contra o alvo;
+    - O bônus é cumulativo até o máximo de +5;
+    - Caso falhe em uma ação contra o alvo, perde todo o bônus acumulado.
+- Esse efeito pode ser utilizado em apenas um alvo por vez e permanece até o fim da cena ou combate.
+</t>
   </si>
   <si>
     <t>OLHOS DE BELPHEGOR</t>

</xml_diff>